<commit_message>
fix(proforma): al generar usar la cantidad real del producto y la fecha de emision
</commit_message>
<xml_diff>
--- a/GeneradorProforma/src/GeneradorProforma.Core/Resources/Plantillas/plantilla.xlsx
+++ b/GeneradorProforma/src/GeneradorProforma.Core/Resources/Plantillas/plantilla.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qwe\source\repos\ConsoleApp1\ConsoleApp1\bin\Debug\net10.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qwe\Documents\personal\senati\projects\practicas\sys_proforma\GeneradorProforma\src\GeneradorProforma.Core\Resources\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E274DED6-FF73-4FF2-888C-BED9B9AEF0D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6315024-6CAE-4D97-87B3-D9E906734B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -117,9 +117,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-  </numFmts>
   <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -488,9 +485,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -525,6 +519,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3876,22 +3871,22 @@
   <sheetData>
     <row r="1" spans="1:8" ht="120" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:8" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
     </row>
     <row r="3" spans="1:8" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
       <c r="D3" s="16" t="s">
         <v>14</v>
       </c>
@@ -3904,7 +3899,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="31"/>
-      <c r="C4" s="53"/>
+      <c r="C4" s="52"/>
       <c r="D4" s="4" t="s">
         <v>11</v>
       </c>
@@ -3916,8 +3911,8 @@
       <c r="A5" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="55"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="54"/>
       <c r="D5" s="31" t="s">
         <v>0</v>
       </c>
@@ -3937,25 +3932,25 @@
       <c r="G6" s="5"/>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="57" t="s">
+      <c r="A7" s="56" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="57" t="s">
+      <c r="C7" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="57" t="s">
+      <c r="D7" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="57" t="s">
+      <c r="E7" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="59" t="s">
+      <c r="F7" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="58" t="s">
+      <c r="G7" s="57" t="s">
         <v>7</v>
       </c>
     </row>
@@ -3967,7 +3962,7 @@
       <c r="C8" s="50"/>
       <c r="D8" s="45"/>
       <c r="E8" s="45"/>
-      <c r="F8" s="52"/>
+      <c r="F8" s="38"/>
       <c r="G8" s="27"/>
       <c r="H8" s="48"/>
     </row>
@@ -3979,7 +3974,7 @@
       <c r="C9" s="50"/>
       <c r="D9" s="45"/>
       <c r="E9" s="45"/>
-      <c r="F9" s="52"/>
+      <c r="F9" s="38"/>
       <c r="G9" s="27"/>
     </row>
     <row r="10" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.25">
@@ -3990,7 +3985,7 @@
       <c r="C10" s="50"/>
       <c r="D10" s="45"/>
       <c r="E10" s="45"/>
-      <c r="F10" s="52"/>
+      <c r="F10" s="38"/>
       <c r="G10" s="27"/>
       <c r="H10" s="48"/>
     </row>
@@ -4002,7 +3997,7 @@
       <c r="C11" s="50"/>
       <c r="D11" s="45"/>
       <c r="E11" s="45"/>
-      <c r="F11" s="52"/>
+      <c r="F11" s="38"/>
       <c r="G11" s="27"/>
       <c r="H11" s="48"/>
     </row>
@@ -4256,7 +4251,7 @@
       <c r="C34" s="29"/>
       <c r="D34" s="29"/>
       <c r="E34" s="29"/>
-      <c r="F34" s="29"/>
+      <c r="F34" s="64"/>
       <c r="G34" s="27"/>
     </row>
     <row r="35" spans="1:7" s="10" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -4278,7 +4273,7 @@
       <c r="C36" s="30"/>
       <c r="D36" s="29"/>
       <c r="E36" s="29"/>
-      <c r="F36" s="29"/>
+      <c r="F36" s="64"/>
       <c r="G36" s="27"/>
     </row>
     <row r="37" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -4289,7 +4284,7 @@
       <c r="C37" s="30"/>
       <c r="D37" s="29"/>
       <c r="E37" s="29"/>
-      <c r="F37" s="29"/>
+      <c r="F37" s="64"/>
       <c r="G37" s="27"/>
     </row>
     <row r="38" spans="1:7" s="10" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4311,7 +4306,7 @@
     </row>
     <row r="39" spans="1:7" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="56" t="s">
+      <c r="B39" s="55" t="s">
         <v>16</v>
       </c>
       <c r="C39" s="32"/>
@@ -4346,10 +4341,10 @@
         <v>23</v>
       </c>
       <c r="C41" s="34"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="63"/>
-      <c r="F41" s="63"/>
-      <c r="G41" s="63"/>
+      <c r="D41" s="62"/>
+      <c r="E41" s="62"/>
+      <c r="F41" s="62"/>
+      <c r="G41" s="62"/>
     </row>
     <row r="42" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="13"/>
@@ -4401,12 +4396,12 @@
       <c r="A47"/>
       <c r="B47"/>
       <c r="C47" s="1"/>
-      <c r="D47" s="64" t="s">
+      <c r="D47" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="E47" s="64"/>
-      <c r="F47" s="64"/>
-      <c r="G47" s="64"/>
+      <c r="E47" s="63"/>
+      <c r="F47" s="63"/>
+      <c r="G47" s="63"/>
     </row>
     <row r="48" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48"/>
@@ -4420,15 +4415,15 @@
       <c r="G48" s="1"/>
     </row>
     <row r="49" spans="1:7" s="10" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A49" s="62" t="s">
+      <c r="A49" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="B49" s="62"/>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
+      <c r="B49" s="61"/>
+      <c r="C49" s="61"/>
+      <c r="D49" s="61"/>
+      <c r="E49" s="61"/>
+      <c r="F49" s="61"/>
+      <c r="G49" s="61"/>
     </row>
     <row r="50" spans="1:7" s="10" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="D50" s="6"/>

</xml_diff>